<commit_message>
modificando la relación ResinteInmueble 0001 del modelo de dominio anemico
</commit_message>
<xml_diff>
--- a/Doo-Doc/Nueva Version Victus/Modelo de dominio anémico/Modelo de dominio anémico de contextos-VictusResidencias.xlsx
+++ b/Doo-Doc/Nueva Version Victus/Modelo de dominio anémico/Modelo de dominio anémico de contextos-VictusResidencias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\josez\Documents\Universidad IngeSistemas\Diseño Orientado a Objetos(DOO)\VictusProyect\victus-doc\Doo-Doc\Nueva Version Victus\Modelo de dominio anémico\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\DOO 2024 BD\DOO\victus-doc\Doo-Doc\Nueva Version Victus\Modelo de dominio anémico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4420D9F7-73E8-441A-B51F-74BACC928EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BDE411C-CB91-4771-87FC-995C82F464A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="9" xr2:uid="{082AFB46-52C9-4E4C-AE4E-19443AA1B53B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="5" xr2:uid="{082AFB46-52C9-4E4C-AE4E-19443AA1B53B}"/>
   </bookViews>
   <sheets>
     <sheet name="Valores" sheetId="3" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="101">
   <si>
     <t>Problema/Dominio:</t>
   </si>
@@ -321,9 +321,6 @@
     <t>fechaHoraInicio</t>
   </si>
   <si>
-    <t>NombreAgenda</t>
-  </si>
-  <si>
     <t>Atributo que contiene la información del identificador de una zona común en el contexto de Conjuntos Residenciales</t>
   </si>
   <si>
@@ -336,15 +333,6 @@
     <t>Entero</t>
   </si>
   <si>
-    <t>Atributo que contiene la información del identificador de un inmueble en el contexto de Conjuntos Residenciales</t>
-  </si>
-  <si>
-    <t>tipoZonaInmueble</t>
-  </si>
-  <si>
-    <t>numeroZonaInmueble</t>
-  </si>
-  <si>
     <t>fechaHoraFin</t>
   </si>
   <si>
@@ -358,6 +346,9 @@
   </si>
   <si>
     <t>unidadTiempoUso</t>
+  </si>
+  <si>
+    <t>TipoInmueble</t>
   </si>
 </sst>
 </file>
@@ -410,7 +401,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -483,8 +474,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="46">
+  <borders count="41">
     <border>
       <left/>
       <right/>
@@ -926,30 +923,63 @@
       <right style="thick">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
         <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
+      <left/>
+      <right style="thick">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
@@ -957,108 +987,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thick">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top style="thick">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
         <color indexed="64"/>
       </right>
       <top/>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top style="thick">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thick">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top style="thick">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thick">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -1068,7 +1002,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="147">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1226,6 +1160,21 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1349,6 +1298,78 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1364,154 +1385,61 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1951,10 +1879,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="54"/>
+      <c r="B1" s="59"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
@@ -2081,75 +2009,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="101" t="str">
+      <c r="B1" s="99" t="str">
         <f>Reservas!D8</f>
         <v>Reserva-0001</v>
       </c>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="102"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="99"/>
+      <c r="L1" s="99"/>
+      <c r="M1" s="99"/>
+      <c r="N1" s="99"/>
+      <c r="O1" s="99"/>
+      <c r="P1" s="99"/>
+      <c r="Q1" s="99"/>
+      <c r="R1" s="99"/>
+      <c r="S1" s="100"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="89"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="90"/>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="90"/>
-      <c r="Q2" s="90"/>
-      <c r="R2" s="90"/>
-      <c r="S2" s="91"/>
+      <c r="A2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="95"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="96"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="101" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="104"/>
-      <c r="C3" s="104"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104" t="s">
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="104"/>
-      <c r="L3" s="104"/>
-      <c r="M3" s="104"/>
-      <c r="N3" s="104"/>
-      <c r="O3" s="104"/>
-      <c r="P3" s="104"/>
-      <c r="Q3" s="104"/>
-      <c r="R3" s="105" t="s">
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="102"/>
+      <c r="O3" s="102"/>
+      <c r="P3" s="102"/>
+      <c r="Q3" s="102"/>
+      <c r="R3" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="107" t="s">
+      <c r="S3" s="105" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2205,14 +2133,14 @@
       <c r="Q4" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="R4" s="106"/>
-      <c r="S4" s="108"/>
+      <c r="R4" s="120"/>
+      <c r="S4" s="106"/>
     </row>
     <row r="5" spans="1:19" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="94" t="s">
+      <c r="A5" s="123" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="97" t="s">
+      <c r="B5" s="126" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="51" t="s">
@@ -2249,17 +2177,17 @@
       <c r="O5" s="51"/>
       <c r="P5" s="51"/>
       <c r="Q5" s="51"/>
-      <c r="R5" s="137" t="s">
-        <v>92</v>
-      </c>
-      <c r="S5" s="110" t="str">
+      <c r="R5" s="112" t="s">
+        <v>91</v>
+      </c>
+      <c r="S5" s="114" t="str">
         <f>B11</f>
         <v>Turno</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="95"/>
-      <c r="B6" s="98"/>
+      <c r="A6" s="124"/>
+      <c r="B6" s="127"/>
       <c r="C6" s="51" t="s">
         <v>4</v>
       </c>
@@ -2294,12 +2222,12 @@
       <c r="O6" s="51"/>
       <c r="P6" s="51"/>
       <c r="Q6" s="51"/>
-      <c r="R6" s="138"/>
-      <c r="S6" s="111"/>
+      <c r="R6" s="113"/>
+      <c r="S6" s="115"/>
     </row>
     <row r="7" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="95"/>
-      <c r="B7" s="114" t="s">
+      <c r="A7" s="124"/>
+      <c r="B7" s="128" t="s">
         <v>64</v>
       </c>
       <c r="C7" s="50" t="s">
@@ -2340,11 +2268,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B7,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Agenda  en el contexto de Agendas.</v>
       </c>
-      <c r="S7" s="111"/>
+      <c r="S7" s="115"/>
     </row>
     <row r="8" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="95"/>
-      <c r="B8" s="115"/>
+      <c r="A8" s="124"/>
+      <c r="B8" s="129"/>
       <c r="C8" s="50" t="s">
         <v>4</v>
       </c>
@@ -2380,13 +2308,13 @@
       <c r="P8" s="31"/>
       <c r="Q8" s="31"/>
       <c r="R8" s="40" t="s">
-        <v>100</v>
-      </c>
-      <c r="S8" s="111"/>
+        <v>96</v>
+      </c>
+      <c r="S8" s="115"/>
     </row>
     <row r="9" spans="1:19" ht="58.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="95"/>
-      <c r="B9" s="115"/>
+      <c r="A9" s="124"/>
+      <c r="B9" s="129"/>
       <c r="C9" s="31" t="s">
         <v>90</v>
       </c>
@@ -2417,13 +2345,13 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B7," en el contexto de ",A5," asociado al residente con el identificador' ",J9,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Agenda en el contexto de Agendas asociado al residente con el identificador' fechaHoraInicioAgenda'.</v>
       </c>
-      <c r="S9" s="111"/>
+      <c r="S9" s="115"/>
     </row>
     <row r="10" spans="1:19" ht="58.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="95"/>
-      <c r="B10" s="99"/>
+      <c r="A10" s="124"/>
+      <c r="B10" s="130"/>
       <c r="C10" s="31" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D10" s="31" t="s">
         <v>58</v>
@@ -2452,11 +2380,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B8," en el contexto de ",A6," asociado al residente con el identificador' ",J10,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' fechaHoraFinAgenda'.</v>
       </c>
-      <c r="S10" s="111"/>
+      <c r="S10" s="115"/>
     </row>
     <row r="11" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="95"/>
-      <c r="B11" s="100" t="s">
+      <c r="A11" s="124"/>
+      <c r="B11" s="122" t="s">
         <v>65</v>
       </c>
       <c r="C11" s="32" t="s">
@@ -2497,11 +2425,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B11,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Turno  en el contexto de Agendas.</v>
       </c>
-      <c r="S11" s="111"/>
+      <c r="S11" s="115"/>
     </row>
     <row r="12" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="95"/>
-      <c r="B12" s="100"/>
+      <c r="A12" s="124"/>
+      <c r="B12" s="122"/>
       <c r="C12" s="32" t="s">
         <v>57</v>
       </c>
@@ -2540,11 +2468,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B11," en el contexto de ",A5," asociado a la reserva con el identificador' ",J12,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Turno en el contexto de Agendas asociado a la reserva con el identificador' NombreTurno'.</v>
       </c>
-      <c r="S12" s="111"/>
+      <c r="S12" s="115"/>
     </row>
     <row r="13" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="96"/>
-      <c r="B13" s="100"/>
+      <c r="A13" s="125"/>
+      <c r="B13" s="122"/>
       <c r="C13" s="32" t="s">
         <v>62</v>
       </c>
@@ -2568,7 +2496,7 @@
       <c r="P13" s="32"/>
       <c r="Q13" s="32"/>
       <c r="R13" s="41"/>
-      <c r="S13" s="112"/>
+      <c r="S13" s="121"/>
     </row>
     <row r="14" spans="1:19" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -2621,75 +2549,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="101" t="str">
+      <c r="B1" s="99" t="str">
         <f>Reservas!D8</f>
         <v>Reserva-0001</v>
       </c>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="102"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="99"/>
+      <c r="L1" s="99"/>
+      <c r="M1" s="99"/>
+      <c r="N1" s="99"/>
+      <c r="O1" s="99"/>
+      <c r="P1" s="99"/>
+      <c r="Q1" s="99"/>
+      <c r="R1" s="99"/>
+      <c r="S1" s="100"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="89"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="90"/>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="90"/>
-      <c r="Q2" s="90"/>
-      <c r="R2" s="90"/>
-      <c r="S2" s="91"/>
+      <c r="A2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="95"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="96"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="101" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="104"/>
-      <c r="C3" s="104"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104" t="s">
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="104"/>
-      <c r="L3" s="104"/>
-      <c r="M3" s="104"/>
-      <c r="N3" s="104"/>
-      <c r="O3" s="104"/>
-      <c r="P3" s="104"/>
-      <c r="Q3" s="104"/>
-      <c r="R3" s="105" t="s">
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="102"/>
+      <c r="O3" s="102"/>
+      <c r="P3" s="102"/>
+      <c r="Q3" s="102"/>
+      <c r="R3" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="107" t="s">
+      <c r="S3" s="105" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2745,14 +2673,14 @@
       <c r="Q4" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="R4" s="113"/>
-      <c r="S4" s="108"/>
+      <c r="R4" s="104"/>
+      <c r="S4" s="106"/>
     </row>
     <row r="5" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="109" t="s">
+      <c r="A5" s="131" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="139" t="s">
+      <c r="B5" s="132" t="s">
         <v>82</v>
       </c>
       <c r="C5" s="31" t="s">
@@ -2793,16 +2721,16 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B5,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Inmueble  en el contexto de Residentes.</v>
       </c>
-      <c r="S5" s="110" t="str">
+      <c r="S5" s="114" t="str">
         <f>B8</f>
         <v>Residente</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="109"/>
-      <c r="B6" s="140"/>
+      <c r="A6" s="131"/>
+      <c r="B6" s="133"/>
       <c r="C6" s="31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D6" s="31" t="s">
         <v>58</v>
@@ -2839,16 +2767,16 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B5," en el contexto de ",A5," asociado al residente con el identificador' ",J6,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Inmueble en el contexto de Residentes asociado al residente con el identificador' tipoInmuebleInmueble'.</v>
       </c>
-      <c r="S6" s="111"/>
+      <c r="S6" s="115"/>
     </row>
     <row r="7" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="109"/>
-      <c r="B7" s="141"/>
+      <c r="A7" s="131"/>
+      <c r="B7" s="134"/>
       <c r="C7" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="31" t="s">
         <v>94</v>
-      </c>
-      <c r="D7" s="31" t="s">
-        <v>95</v>
       </c>
       <c r="E7" s="31">
         <v>1</v>
@@ -2882,11 +2810,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B6," en el contexto de ",A6," asociado al residente con el identificador' ",J7,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' numeroViviendaInmueble'.</v>
       </c>
-      <c r="S7" s="111"/>
+      <c r="S7" s="115"/>
     </row>
     <row r="8" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="109"/>
-      <c r="B8" s="100" t="s">
+      <c r="A8" s="131"/>
+      <c r="B8" s="122" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="32" t="s">
@@ -2927,11 +2855,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B8,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Residente  en el contexto de Residentes.</v>
       </c>
-      <c r="S8" s="111"/>
+      <c r="S8" s="115"/>
     </row>
     <row r="9" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="109"/>
-      <c r="B9" s="100"/>
+      <c r="A9" s="131"/>
+      <c r="B9" s="122"/>
       <c r="C9" s="32" t="s">
         <v>57</v>
       </c>
@@ -2970,7 +2898,7 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B8," en el contexto de ",A5," asociado a la reserva con el identificador' ",J9,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Residente en el contexto de Residentes asociado a la reserva con el identificador' tipoInmuebleResidente'.</v>
       </c>
-      <c r="S9" s="112"/>
+      <c r="S9" s="121"/>
     </row>
     <row r="10" spans="1:19" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -3015,29 +2943,29 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64" t="s">
+      <c r="B1" s="69" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="65"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="70"/>
     </row>
     <row r="2" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="67"/>
-      <c r="D2" s="68"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="73"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="69" t="s">
+      <c r="A3" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="70"/>
-      <c r="D3" s="71"/>
+      <c r="B3" s="75"/>
+      <c r="C3" s="75"/>
+      <c r="D3" s="76"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -3054,132 +2982,132 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="B5" s="80" t="s">
         <v>79</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="76" t="s">
+      <c r="D5" s="81" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="74"/>
-      <c r="B6" s="75"/>
+      <c r="A6" s="79"/>
+      <c r="B6" s="80"/>
       <c r="C6" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="76"/>
+      <c r="D6" s="81"/>
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="74"/>
-      <c r="B7" s="75"/>
+      <c r="A7" s="79"/>
+      <c r="B7" s="80"/>
       <c r="C7" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="76"/>
+      <c r="D7" s="81"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="74"/>
-      <c r="B8" s="75"/>
+      <c r="A8" s="79"/>
+      <c r="B8" s="80"/>
       <c r="C8" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="76"/>
+      <c r="D8" s="81"/>
     </row>
     <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="74"/>
-      <c r="B9" s="75"/>
+      <c r="A9" s="79"/>
+      <c r="B9" s="80"/>
       <c r="C9" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="D9" s="76"/>
+      <c r="D9" s="81"/>
     </row>
     <row r="10" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="72" t="s">
+      <c r="A10" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="73" t="s">
+      <c r="B10" s="78" t="s">
         <v>80</v>
       </c>
       <c r="C10" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="72" t="s">
+      <c r="D10" s="77" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="72"/>
-      <c r="B11" s="73"/>
+      <c r="A11" s="77"/>
+      <c r="B11" s="78"/>
       <c r="C11" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="D11" s="72"/>
+      <c r="D11" s="77"/>
     </row>
     <row r="12" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="80" t="s">
+      <c r="A12" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="77" t="s">
+      <c r="B12" s="82" t="s">
         <v>83</v>
       </c>
       <c r="C12" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="80" t="s">
+      <c r="D12" s="85" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="81"/>
-      <c r="B13" s="78"/>
+      <c r="A13" s="86"/>
+      <c r="B13" s="83"/>
       <c r="C13" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="81"/>
+      <c r="D13" s="86"/>
     </row>
     <row r="14" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="82"/>
-      <c r="B14" s="79"/>
+      <c r="A14" s="87"/>
+      <c r="B14" s="84"/>
       <c r="C14" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="82"/>
+      <c r="D14" s="87"/>
     </row>
     <row r="15" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="55" t="s">
+      <c r="A15" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="63" t="s">
         <v>63</v>
       </c>
       <c r="C15" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="61" t="s">
+      <c r="D15" s="66" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="56"/>
-      <c r="B16" s="59"/>
+      <c r="A16" s="61"/>
+      <c r="B16" s="64"/>
       <c r="C16" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="62"/>
+      <c r="D16" s="67"/>
     </row>
     <row r="17" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="57"/>
-      <c r="B17" s="60"/>
+      <c r="A17" s="62"/>
+      <c r="B17" s="65"/>
       <c r="C17" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="63"/>
+      <c r="D17" s="68"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -3251,50 +3179,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="83" t="str">
+      <c r="B1" s="88" t="str">
         <f>Contextos!B5</f>
         <v xml:space="preserve"> Conjuntos residenciales</v>
       </c>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="84"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="85" t="str">
+      <c r="B2" s="90" t="str">
         <f>Contextos!D5</f>
         <v>Contexto cuya motivación es Gestionar la estructura física y los recursos disponibles en cada conjunto residencial. Aquí se manejan los datos sobre qué conjuntos existen, dónde están ubicados, qué recursos ofrecen según una Agenda con respectivos turnos para cada zona.</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="86"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="91"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="87" t="str">
+      <c r="B3" s="92" t="str">
         <f>Contextos!A5</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="88"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="93"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="91"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="95"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="96"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -3303,14 +3231,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="92" t="s">
+      <c r="C5" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="92" t="s">
+      <c r="D5" s="97" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="92"/>
-      <c r="F5" s="93" t="s">
+      <c r="E5" s="97"/>
+      <c r="F5" s="98" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3321,10 +3249,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
-      <c r="E6" s="92"/>
-      <c r="F6" s="93"/>
+      <c r="C6" s="97"/>
+      <c r="D6" s="97"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="98"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -3333,14 +3261,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="92"/>
+      <c r="C7" s="97"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="93"/>
+      <c r="F7" s="98"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
@@ -3474,50 +3402,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="83" t="str">
+      <c r="B1" s="88" t="str">
         <f>Contextos!B10</f>
         <v>Residentes</v>
       </c>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="84"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="85" t="str">
+      <c r="B2" s="90" t="str">
         <f>Contextos!D10</f>
         <v>Contexto cuya motivación es encargarce de manejar la información de los residentes, incluidas sus identificaciones, contacto, y la relación entre el residente y su residencia dentro del conjunto.</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="86"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="91"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="87" t="str">
+      <c r="B3" s="92" t="str">
         <f>Contextos!A10</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="88"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="93"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="91"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="95"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="96"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -3526,14 +3454,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="92" t="s">
+      <c r="C5" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="92" t="s">
+      <c r="D5" s="97" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="92"/>
-      <c r="F5" s="93" t="s">
+      <c r="E5" s="97"/>
+      <c r="F5" s="98" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3544,10 +3472,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
-      <c r="E6" s="92"/>
-      <c r="F6" s="93"/>
+      <c r="C6" s="97"/>
+      <c r="D6" s="97"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="98"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -3556,14 +3484,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="92"/>
+      <c r="C7" s="97"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="93"/>
+      <c r="F7" s="98"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
@@ -3618,7 +3546,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59635CF3-0DE6-45E6-A198-1E7042F5E8F9}">
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" style="13" bestFit="1" customWidth="1"/>
@@ -3647,75 +3575,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="101" t="str">
+      <c r="B1" s="99" t="str">
         <f>Residentes!D8</f>
         <v>Residente Inmueble-0001</v>
       </c>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="102"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="99"/>
+      <c r="L1" s="99"/>
+      <c r="M1" s="99"/>
+      <c r="N1" s="99"/>
+      <c r="O1" s="99"/>
+      <c r="P1" s="99"/>
+      <c r="Q1" s="99"/>
+      <c r="R1" s="99"/>
+      <c r="S1" s="100"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="89"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="90"/>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="90"/>
-      <c r="Q2" s="90"/>
-      <c r="R2" s="90"/>
-      <c r="S2" s="91"/>
+      <c r="A2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="95"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="96"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="101" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="104"/>
-      <c r="C3" s="104"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104" t="s">
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="104"/>
-      <c r="L3" s="104"/>
-      <c r="M3" s="104"/>
-      <c r="N3" s="104"/>
-      <c r="O3" s="104"/>
-      <c r="P3" s="104"/>
-      <c r="Q3" s="104"/>
-      <c r="R3" s="105" t="s">
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="102"/>
+      <c r="O3" s="102"/>
+      <c r="P3" s="102"/>
+      <c r="Q3" s="102"/>
+      <c r="R3" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="107" t="s">
+      <c r="S3" s="105" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3771,340 +3699,331 @@
       <c r="Q4" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="R4" s="113"/>
-      <c r="S4" s="108"/>
-    </row>
-    <row r="5" spans="1:19" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="134" t="s">
+      <c r="R4" s="104"/>
+      <c r="S4" s="106"/>
+    </row>
+    <row r="5" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="108" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="129" t="s">
+      <c r="B5" s="140" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="51" t="s">
-        <v>55</v>
+      <c r="C5" s="139" t="s">
+        <v>93</v>
       </c>
       <c r="D5" s="51" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="E5" s="51">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="F5" s="51">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="G5" s="51"/>
       <c r="H5" s="51"/>
       <c r="I5" s="51"/>
       <c r="J5" s="51" t="str">
         <f>_xlfn.CONCAT(C5,$B$5)</f>
-        <v>identificadorInmueble</v>
+        <v>numeroViviendaInmueble</v>
       </c>
       <c r="K5" s="51" t="s">
         <v>59</v>
       </c>
       <c r="L5" s="51" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="M5" s="51">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="N5" s="51">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O5" s="51"/>
       <c r="P5" s="51"/>
       <c r="Q5" s="52"/>
-      <c r="R5" s="118" t="s">
-        <v>96</v>
-      </c>
-      <c r="S5" s="119" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="135"/>
-      <c r="B6" s="130"/>
-      <c r="C6" s="51" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" s="51" t="s">
+      <c r="R5" s="143" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C5," del objeto dominio ",B5,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del numeroVivienda del objeto dominio Inmueble  en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S5" s="141" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="108"/>
+      <c r="B6" s="110" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="50" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="31">
+        <v>32</v>
+      </c>
+      <c r="F6" s="31">
+        <v>32</v>
+      </c>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="31" t="str">
+        <f>_xlfn.CONCAT(C6,$B$6)</f>
+        <v>identificadorTipoInmueble</v>
+      </c>
+      <c r="K6" s="31" t="s">
+        <v>59</v>
+      </c>
+      <c r="L6" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="M6" s="31">
+        <v>32</v>
+      </c>
+      <c r="N6" s="31">
+        <v>32</v>
+      </c>
+      <c r="O6" s="31"/>
+      <c r="P6" s="31"/>
+      <c r="Q6" s="53"/>
+      <c r="R6" s="144" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C6," del objeto dominio ",B6,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del identificador del objeto dominio TipoInmueble  en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S6" s="141"/>
+    </row>
+    <row r="7" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="108"/>
+      <c r="B7" s="110"/>
+      <c r="C7" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="51">
+      <c r="E7" s="31">
         <v>1</v>
       </c>
-      <c r="F6" s="51">
-        <v>20</v>
-      </c>
-      <c r="G6" s="51"/>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51" t="str">
-        <f t="shared" ref="J6:J7" si="0">_xlfn.CONCAT(C6,$B$5)</f>
-        <v>tipoInmuebleInmueble</v>
-      </c>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="51"/>
-      <c r="O6" s="51"/>
-      <c r="P6" s="51"/>
-      <c r="Q6" s="52"/>
-      <c r="R6" s="120"/>
-      <c r="S6" s="121"/>
-    </row>
-    <row r="7" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="135"/>
-      <c r="B7" s="131"/>
-      <c r="C7" s="51" t="s">
-        <v>94</v>
-      </c>
-      <c r="D7" s="51" t="s">
-        <v>95</v>
-      </c>
-      <c r="E7" s="51">
+      <c r="F7" s="31">
+        <v>50</v>
+      </c>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="31" t="str">
+        <f>_xlfn.CONCAT(C7,$B$6)</f>
+        <v>nombreTipoInmueble</v>
+      </c>
+      <c r="K7" s="31"/>
+      <c r="L7" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="M7" s="31">
         <v>1</v>
       </c>
-      <c r="F7" s="51">
+      <c r="N7" s="31">
         <v>50</v>
       </c>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="51"/>
-      <c r="J7" s="51" t="str">
-        <f t="shared" si="0"/>
-        <v>numeroViviendaInmueble</v>
-      </c>
-      <c r="K7" s="51" t="s">
+      <c r="O7" s="31"/>
+      <c r="P7" s="31"/>
+      <c r="Q7" s="53"/>
+      <c r="R7" s="144" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C7," del objeto dominio ",B7,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del nombre del objeto dominio   en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S7" s="141"/>
+    </row>
+    <row r="8" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="108"/>
+      <c r="B8" s="135" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="136" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="137" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="137">
+        <v>32</v>
+      </c>
+      <c r="F8" s="137">
+        <v>32</v>
+      </c>
+      <c r="G8" s="137"/>
+      <c r="H8" s="137"/>
+      <c r="I8" s="137"/>
+      <c r="J8" s="137" t="str">
+        <f>_xlfn.CONCAT(C8,$B$6)</f>
+        <v>identificadorTipoInmueble</v>
+      </c>
+      <c r="K8" s="137" t="s">
         <v>59</v>
       </c>
-      <c r="L7" s="51" t="s">
-        <v>95</v>
-      </c>
-      <c r="M7" s="51">
+      <c r="L8" s="137" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" s="137">
+        <v>32</v>
+      </c>
+      <c r="N8" s="137">
+        <v>32</v>
+      </c>
+      <c r="O8" s="137"/>
+      <c r="P8" s="137"/>
+      <c r="Q8" s="138"/>
+      <c r="R8" s="145" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C8," del objeto dominio ",B8,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del identificador del objeto dominio ZonaInmueble  en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S8" s="141"/>
+    </row>
+    <row r="9" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="108"/>
+      <c r="B9" s="135"/>
+      <c r="C9" s="136" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="137" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" s="137">
         <v>1</v>
       </c>
-      <c r="N7" s="51">
+      <c r="F9" s="137">
         <v>50</v>
       </c>
-      <c r="O7" s="51"/>
-      <c r="P7" s="51"/>
-      <c r="Q7" s="52"/>
-      <c r="R7" s="122"/>
-      <c r="S7" s="121"/>
-    </row>
-    <row r="8" spans="1:19" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="135"/>
-      <c r="B8" s="132" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="50" t="s">
+      <c r="G9" s="137"/>
+      <c r="H9" s="137"/>
+      <c r="I9" s="137"/>
+      <c r="J9" s="137" t="str">
+        <f>_xlfn.CONCAT(C9,$B$6)</f>
+        <v>nombreTipoInmueble</v>
+      </c>
+      <c r="K9" s="137"/>
+      <c r="L9" s="137" t="s">
+        <v>58</v>
+      </c>
+      <c r="M9" s="137">
+        <v>1</v>
+      </c>
+      <c r="N9" s="137">
+        <v>50</v>
+      </c>
+      <c r="O9" s="137"/>
+      <c r="P9" s="137"/>
+      <c r="Q9" s="138"/>
+      <c r="R9" s="145" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C9," del objeto dominio ",B9,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del nombre del objeto dominio   en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S9" s="141"/>
+    </row>
+    <row r="10" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="108"/>
+      <c r="B10" s="111" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="31" t="s">
+      <c r="D10" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="31">
+      <c r="E10" s="32">
         <v>32</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F10" s="32">
         <v>32</v>
       </c>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="31" t="str">
-        <f>_xlfn.CONCAT(C8,$B$8)</f>
-        <v>identificadorZonaInmueble</v>
-      </c>
-      <c r="K8" s="31" t="s">
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="32" t="str">
+        <f>_xlfn.CONCAT(C6,$B$10)</f>
+        <v>identificadorConjuntoResidencial</v>
+      </c>
+      <c r="K10" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="L8" s="31" t="s">
+      <c r="L10" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="M8" s="31">
+      <c r="M10" s="32">
         <v>32</v>
       </c>
-      <c r="N8" s="31">
+      <c r="N10" s="32">
         <v>32</v>
       </c>
-      <c r="O8" s="31"/>
-      <c r="P8" s="31"/>
-      <c r="Q8" s="116"/>
-      <c r="R8" s="123" t="str">
-        <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B8,"  en el contexto de ",A5,".")</f>
-        <v>Atributo que contiene la informacion del identificador de un ZonaInmueble  en el contexto de Conjuntos Residenciales.</v>
-      </c>
-      <c r="S8" s="121"/>
-    </row>
-    <row r="9" spans="1:19" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="135"/>
-      <c r="B9" s="132"/>
-      <c r="C9" s="50" t="s">
-        <v>97</v>
-      </c>
-      <c r="D9" s="31" t="s">
+      <c r="O10" s="32"/>
+      <c r="P10" s="32"/>
+      <c r="Q10" s="54"/>
+      <c r="R10" s="146" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C10," del objeto dominio ",B10,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del identificador del objeto dominio ConjuntoResidencial  en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S10" s="141"/>
+    </row>
+    <row r="11" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="109"/>
+      <c r="B11" s="111"/>
+      <c r="C11" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="31">
-        <v>5</v>
-      </c>
-      <c r="F9" s="31">
-        <v>6</v>
-      </c>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31" t="str">
-        <f>_xlfn.CONCAT(C9,$B$8)</f>
-        <v>tipoZonaInmuebleZonaInmueble</v>
-      </c>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="31"/>
-      <c r="P9" s="31"/>
-      <c r="Q9" s="116"/>
-      <c r="R9" s="124"/>
-      <c r="S9" s="121"/>
-    </row>
-    <row r="10" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="135"/>
-      <c r="B10" s="132"/>
-      <c r="C10" s="50" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" s="31">
+      <c r="E11" s="32">
         <v>1</v>
       </c>
-      <c r="F10" s="31">
-        <v>30</v>
-      </c>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31" t="s">
-        <v>91</v>
-      </c>
-      <c r="K10" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="L10" s="31"/>
-      <c r="M10" s="31"/>
-      <c r="N10" s="31"/>
-      <c r="O10" s="31"/>
-      <c r="P10" s="31"/>
-      <c r="Q10" s="116"/>
-      <c r="R10" s="125"/>
-      <c r="S10" s="121"/>
-    </row>
-    <row r="11" spans="1:19" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="135"/>
-      <c r="B11" s="133" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="32" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="32">
-        <v>32</v>
-      </c>
       <c r="F11" s="32">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="G11" s="32"/>
       <c r="H11" s="32"/>
       <c r="I11" s="32"/>
       <c r="J11" s="32" t="str">
-        <f>_xlfn.CONCAT(C8,$B$11)</f>
-        <v>identificadorConjuntoResidencial</v>
+        <f>_xlfn.CONCAT(C7,$B$10)</f>
+        <v>nombreConjuntoResidencial</v>
       </c>
       <c r="K11" s="32" t="s">
         <v>59</v>
       </c>
       <c r="L11" s="32" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="M11" s="32">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="N11" s="32">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="O11" s="32"/>
       <c r="P11" s="32"/>
-      <c r="Q11" s="117"/>
-      <c r="R11" s="126" t="str">
-        <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B11,"  en el contexto de ",A5,".")</f>
-        <v>Atributo que contiene la informacion del identificador de un ConjuntoResidencial  en el contexto de Conjuntos Residenciales.</v>
-      </c>
-      <c r="S11" s="121"/>
-    </row>
-    <row r="12" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="136"/>
-      <c r="B12" s="133"/>
-      <c r="C12" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="32" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="32">
-        <v>1</v>
-      </c>
-      <c r="F12" s="32">
-        <v>50</v>
-      </c>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32" t="str">
-        <f>_xlfn.CONCAT(C9,$B$11)</f>
-        <v>tipoZonaInmuebleConjuntoResidencial</v>
-      </c>
-      <c r="K12" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="L12" s="32" t="s">
-        <v>58</v>
-      </c>
-      <c r="M12" s="32">
-        <v>1</v>
-      </c>
-      <c r="N12" s="32">
-        <v>50</v>
-      </c>
-      <c r="O12" s="32"/>
-      <c r="P12" s="32"/>
-      <c r="Q12" s="117"/>
-      <c r="R12" s="127"/>
-      <c r="S12" s="128"/>
+      <c r="Q11" s="54"/>
+      <c r="R11" s="146" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C11," del objeto dominio ",B11,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del nombre del objeto dominio   en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S11" s="142"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="11">
+    <mergeCell ref="A5:A11"/>
+    <mergeCell ref="S5:S11"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B8:B9"/>
     <mergeCell ref="B1:S1"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="J3:Q3"/>
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
-    <mergeCell ref="A5:A12"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="S5:S12"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="R5:R7"/>
-    <mergeCell ref="R8:R10"/>
-    <mergeCell ref="R11:R12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4127,50 +4046,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="83" t="str">
+      <c r="B1" s="88" t="str">
         <f>Contextos!B12</f>
         <v>Agendas</v>
       </c>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="84"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="85" t="str">
+      <c r="B2" s="90" t="str">
         <f>Contextos!D12</f>
         <v>Contexto cuya motivación es la de gestionar la estructura de la agenda que va a tener una zona común durante un un tiempo estimado y sus diferentes turnos.</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="86"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="91"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="87" t="str">
+      <c r="B3" s="92" t="str">
         <f>Contextos!A12</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="88"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="93"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="91"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="95"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="96"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -4179,14 +4098,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="92" t="s">
+      <c r="C5" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="92" t="s">
+      <c r="D5" s="97" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="92"/>
-      <c r="F5" s="93" t="s">
+      <c r="E5" s="97"/>
+      <c r="F5" s="98" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4197,10 +4116,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
-      <c r="E6" s="92"/>
-      <c r="F6" s="93"/>
+      <c r="C6" s="97"/>
+      <c r="D6" s="97"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="98"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -4209,14 +4128,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="92"/>
+      <c r="C7" s="97"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="93"/>
+      <c r="F7" s="98"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
@@ -4322,75 +4241,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="101" t="str">
+      <c r="B1" s="99" t="str">
         <f>Agendas!D8</f>
         <v>Agenda ZonaComun-0001</v>
       </c>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="102"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
+      <c r="J1" s="99"/>
+      <c r="K1" s="99"/>
+      <c r="L1" s="99"/>
+      <c r="M1" s="99"/>
+      <c r="N1" s="99"/>
+      <c r="O1" s="99"/>
+      <c r="P1" s="99"/>
+      <c r="Q1" s="99"/>
+      <c r="R1" s="99"/>
+      <c r="S1" s="100"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="89"/>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="90"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="90"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
-      <c r="L2" s="90"/>
-      <c r="M2" s="90"/>
-      <c r="N2" s="90"/>
-      <c r="O2" s="90"/>
-      <c r="P2" s="90"/>
-      <c r="Q2" s="90"/>
-      <c r="R2" s="90"/>
-      <c r="S2" s="91"/>
+      <c r="A2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
+      <c r="P2" s="95"/>
+      <c r="Q2" s="95"/>
+      <c r="R2" s="95"/>
+      <c r="S2" s="96"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="103" t="s">
+      <c r="A3" s="101" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="104"/>
-      <c r="C3" s="104"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104" t="s">
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="102"/>
+      <c r="I3" s="102"/>
+      <c r="J3" s="102" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="104"/>
-      <c r="L3" s="104"/>
-      <c r="M3" s="104"/>
-      <c r="N3" s="104"/>
-      <c r="O3" s="104"/>
-      <c r="P3" s="104"/>
-      <c r="Q3" s="104"/>
-      <c r="R3" s="105" t="s">
+      <c r="K3" s="102"/>
+      <c r="L3" s="102"/>
+      <c r="M3" s="102"/>
+      <c r="N3" s="102"/>
+      <c r="O3" s="102"/>
+      <c r="P3" s="102"/>
+      <c r="Q3" s="102"/>
+      <c r="R3" s="103" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="107" t="s">
+      <c r="S3" s="105" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4446,14 +4365,14 @@
       <c r="Q4" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="R4" s="106"/>
-      <c r="S4" s="108"/>
+      <c r="R4" s="120"/>
+      <c r="S4" s="106"/>
     </row>
     <row r="5" spans="1:19" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="134" t="s">
+      <c r="A5" s="107" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="142" t="s">
+      <c r="B5" s="116" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="51" t="s">
@@ -4490,17 +4409,17 @@
       <c r="O5" s="51"/>
       <c r="P5" s="51"/>
       <c r="Q5" s="51"/>
-      <c r="R5" s="137" t="str">
+      <c r="R5" s="112" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B7," en el contexto de ",A5," asociado al residente con el identificador' ",J9,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de Conjuntos Residenciales asociado al residente con el identificador' unidadTiempoUsoZonaComun'.</v>
       </c>
-      <c r="S5" s="110" t="s">
+      <c r="S5" s="114" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="135"/>
-      <c r="B6" s="143"/>
+      <c r="A6" s="108"/>
+      <c r="B6" s="117"/>
       <c r="C6" s="51" t="s">
         <v>4</v>
       </c>
@@ -4535,17 +4454,17 @@
       <c r="O6" s="51"/>
       <c r="P6" s="51"/>
       <c r="Q6" s="51"/>
-      <c r="R6" s="138"/>
-      <c r="S6" s="111"/>
+      <c r="R6" s="113"/>
+      <c r="S6" s="115"/>
     </row>
     <row r="7" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="135"/>
-      <c r="B7" s="143"/>
+      <c r="A7" s="108"/>
+      <c r="B7" s="117"/>
       <c r="C7" s="51" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D7" s="51" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E7" s="51"/>
       <c r="F7" s="51"/>
@@ -4563,20 +4482,20 @@
       <c r="O7" s="51"/>
       <c r="P7" s="51"/>
       <c r="Q7" s="51"/>
-      <c r="R7" s="137" t="str">
+      <c r="R7" s="112" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B9," en el contexto de ",A7," asociado al residente con el identificador' ",J11,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' nombreConjuntoResidencial'.</v>
       </c>
-      <c r="S7" s="111"/>
+      <c r="S7" s="115"/>
     </row>
     <row r="8" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="135"/>
-      <c r="B8" s="143"/>
+      <c r="A8" s="108"/>
+      <c r="B8" s="117"/>
       <c r="C8" s="51" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D8" s="51" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E8" s="51"/>
       <c r="F8" s="51"/>
@@ -4594,14 +4513,14 @@
       <c r="O8" s="51"/>
       <c r="P8" s="51"/>
       <c r="Q8" s="51"/>
-      <c r="R8" s="147"/>
-      <c r="S8" s="111"/>
+      <c r="R8" s="119"/>
+      <c r="S8" s="115"/>
     </row>
     <row r="9" spans="1:19" ht="61.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="135"/>
-      <c r="B9" s="144"/>
+      <c r="A9" s="108"/>
+      <c r="B9" s="118"/>
       <c r="C9" s="51" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D9" s="51" t="s">
         <v>58</v>
@@ -4622,15 +4541,15 @@
       <c r="O9" s="51"/>
       <c r="P9" s="51"/>
       <c r="Q9" s="52"/>
-      <c r="R9" s="148" t="str">
+      <c r="R9" s="57" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B11," en el contexto de ",A9," asociado al residente con el identificador' ",J13,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' '.</v>
       </c>
-      <c r="S9" s="111"/>
+      <c r="S9" s="115"/>
     </row>
     <row r="10" spans="1:19" ht="60.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="135"/>
-      <c r="B10" s="133" t="s">
+      <c r="A10" s="108"/>
+      <c r="B10" s="111" t="s">
         <v>61</v>
       </c>
       <c r="C10" s="32" t="s">
@@ -4666,16 +4585,16 @@
       </c>
       <c r="O10" s="32"/>
       <c r="P10" s="32"/>
-      <c r="Q10" s="117"/>
-      <c r="R10" s="146" t="str">
+      <c r="Q10" s="54"/>
+      <c r="R10" s="56" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B10," en el contexto de ",A10," asociado a la reserva con el identificador' ",J10,"'.")</f>
         <v>Atributo que contiene la información del nombre de un ConjuntoResidencial en el contexto de  asociado a la reserva con el identificador' identificadorConjuntoResidencial'.</v>
       </c>
-      <c r="S10" s="111"/>
+      <c r="S10" s="115"/>
     </row>
     <row r="11" spans="1:19" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="136"/>
-      <c r="B11" s="133"/>
+      <c r="A11" s="109"/>
+      <c r="B11" s="111"/>
       <c r="C11" s="32" t="s">
         <v>57</v>
       </c>
@@ -4710,26 +4629,26 @@
       <c r="O11" s="32"/>
       <c r="P11" s="32"/>
       <c r="Q11" s="32"/>
-      <c r="R11" s="145" t="str">
+      <c r="R11" s="55" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B11," en el contexto de ",A11," asociado a la reserva con el identificador' ",J11,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado a la reserva con el identificador' nombreConjuntoResidencial'.</v>
       </c>
-      <c r="S11" s="111"/>
+      <c r="S11" s="115"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B1:S1"/>
+    <mergeCell ref="A2:S2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="J3:Q3"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="S3:S4"/>
     <mergeCell ref="A5:A11"/>
     <mergeCell ref="R5:R6"/>
     <mergeCell ref="S5:S11"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B5:B9"/>
     <mergeCell ref="R7:R8"/>
-    <mergeCell ref="B1:S1"/>
-    <mergeCell ref="A2:S2"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="J3:Q3"/>
-    <mergeCell ref="R3:R4"/>
-    <mergeCell ref="S3:S4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4753,50 +4672,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="83" t="str">
+      <c r="B1" s="88" t="str">
         <f>Contextos!B15</f>
         <v>Reservas</v>
       </c>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="84"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="85" t="str">
+      <c r="B2" s="90" t="str">
         <f>Contextos!D15</f>
         <v>Contexto cuya intención enfocarse en la gestión del proceso de reservas de los recursos, incluyendo la disponibilidad de los recursos y las reservas que los residentes realizan.</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="86"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="91"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="87" t="str">
+      <c r="B3" s="92" t="str">
         <f>Contextos!A15</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="88"/>
+      <c r="C3" s="92"/>
+      <c r="D3" s="92"/>
+      <c r="E3" s="92"/>
+      <c r="F3" s="93"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="90"/>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="91"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="95"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="96"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -4805,14 +4724,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="92" t="s">
+      <c r="C5" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="92" t="s">
+      <c r="D5" s="97" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="92"/>
-      <c r="F5" s="93" t="s">
+      <c r="E5" s="97"/>
+      <c r="F5" s="98" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4823,10 +4742,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="92"/>
-      <c r="D6" s="92"/>
-      <c r="E6" s="92"/>
-      <c r="F6" s="93"/>
+      <c r="C6" s="97"/>
+      <c r="D6" s="97"/>
+      <c r="E6" s="97"/>
+      <c r="F6" s="98"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -4835,14 +4754,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="92"/>
+      <c r="C7" s="97"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="93"/>
+      <c r="F7" s="98"/>
     </row>
     <row r="8" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">

</xml_diff>

<commit_message>
actualizando residente inmueble 0001 de anemico
</commit_message>
<xml_diff>
--- a/Doo-Doc/Nueva Version Victus/Modelo de dominio anémico/Modelo de dominio anémico de contextos-VictusResidencias.xlsx
+++ b/Doo-Doc/Nueva Version Victus/Modelo de dominio anémico/Modelo de dominio anémico de contextos-VictusResidencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\DOO 2024 BD\DOO\victus-doc\Doo-Doc\Nueva Version Victus\Modelo de dominio anémico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BDE411C-CB91-4771-87FC-995C82F464A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C280229-26CD-4B80-88ED-7C2DB4826BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="5" xr2:uid="{082AFB46-52C9-4E4C-AE4E-19443AA1B53B}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="102">
   <si>
     <t>Problema/Dominio:</t>
   </si>
@@ -349,6 +349,9 @@
   </si>
   <si>
     <t>TipoInmueble</t>
+  </si>
+  <si>
+    <t>TipoZonaInmueble</t>
   </si>
 </sst>
 </file>
@@ -481,7 +484,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -997,12 +1000,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1175,6 +1191,30 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1298,6 +1338,21 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1322,21 +1377,12 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1361,9 +1407,6 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1406,41 +1449,32 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1879,10 +1913,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="66" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="59"/>
+      <c r="B1" s="67"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
@@ -2009,75 +2043,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="99" t="str">
+      <c r="B1" s="112" t="str">
         <f>Reservas!D8</f>
         <v>Reserva-0001</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
-      <c r="R1" s="99"/>
-      <c r="S1" s="100"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
+      <c r="P1" s="112"/>
+      <c r="Q1" s="112"/>
+      <c r="R1" s="112"/>
+      <c r="S1" s="113"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="94"/>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="96"/>
+      <c r="A2" s="102"/>
+      <c r="B2" s="103"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="103"/>
+      <c r="P2" s="103"/>
+      <c r="Q2" s="103"/>
+      <c r="R2" s="103"/>
+      <c r="S2" s="104"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="114" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102" t="s">
+      <c r="B3" s="115"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="103" t="s">
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="105" t="s">
+      <c r="S3" s="118" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2134,13 +2168,13 @@
         <v>52</v>
       </c>
       <c r="R4" s="120"/>
-      <c r="S4" s="106"/>
+      <c r="S4" s="119"/>
     </row>
     <row r="5" spans="1:19" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="123" t="s">
+      <c r="A5" s="132" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="126" t="s">
+      <c r="B5" s="135" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="51" t="s">
@@ -2177,17 +2211,17 @@
       <c r="O5" s="51"/>
       <c r="P5" s="51"/>
       <c r="Q5" s="51"/>
-      <c r="R5" s="112" t="s">
+      <c r="R5" s="122" t="s">
         <v>91</v>
       </c>
-      <c r="S5" s="114" t="str">
+      <c r="S5" s="124" t="str">
         <f>B11</f>
         <v>Turno</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="124"/>
-      <c r="B6" s="127"/>
+      <c r="A6" s="133"/>
+      <c r="B6" s="136"/>
       <c r="C6" s="51" t="s">
         <v>4</v>
       </c>
@@ -2222,12 +2256,12 @@
       <c r="O6" s="51"/>
       <c r="P6" s="51"/>
       <c r="Q6" s="51"/>
-      <c r="R6" s="113"/>
-      <c r="S6" s="115"/>
+      <c r="R6" s="123"/>
+      <c r="S6" s="125"/>
     </row>
     <row r="7" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="124"/>
-      <c r="B7" s="128" t="s">
+      <c r="A7" s="133"/>
+      <c r="B7" s="137" t="s">
         <v>64</v>
       </c>
       <c r="C7" s="50" t="s">
@@ -2268,11 +2302,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B7,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Agenda  en el contexto de Agendas.</v>
       </c>
-      <c r="S7" s="115"/>
+      <c r="S7" s="125"/>
     </row>
     <row r="8" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="124"/>
-      <c r="B8" s="129"/>
+      <c r="A8" s="133"/>
+      <c r="B8" s="138"/>
       <c r="C8" s="50" t="s">
         <v>4</v>
       </c>
@@ -2310,11 +2344,11 @@
       <c r="R8" s="40" t="s">
         <v>96</v>
       </c>
-      <c r="S8" s="115"/>
+      <c r="S8" s="125"/>
     </row>
     <row r="9" spans="1:19" ht="58.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="124"/>
-      <c r="B9" s="129"/>
+      <c r="A9" s="133"/>
+      <c r="B9" s="138"/>
       <c r="C9" s="31" t="s">
         <v>90</v>
       </c>
@@ -2345,11 +2379,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B7," en el contexto de ",A5," asociado al residente con el identificador' ",J9,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Agenda en el contexto de Agendas asociado al residente con el identificador' fechaHoraInicioAgenda'.</v>
       </c>
-      <c r="S9" s="115"/>
+      <c r="S9" s="125"/>
     </row>
     <row r="10" spans="1:19" ht="58.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="124"/>
-      <c r="B10" s="130"/>
+      <c r="A10" s="133"/>
+      <c r="B10" s="139"/>
       <c r="C10" s="31" t="s">
         <v>95</v>
       </c>
@@ -2380,11 +2414,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B8," en el contexto de ",A6," asociado al residente con el identificador' ",J10,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' fechaHoraFinAgenda'.</v>
       </c>
-      <c r="S10" s="115"/>
+      <c r="S10" s="125"/>
     </row>
     <row r="11" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="124"/>
-      <c r="B11" s="122" t="s">
+      <c r="A11" s="133"/>
+      <c r="B11" s="131" t="s">
         <v>65</v>
       </c>
       <c r="C11" s="32" t="s">
@@ -2425,11 +2459,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B11,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Turno  en el contexto de Agendas.</v>
       </c>
-      <c r="S11" s="115"/>
+      <c r="S11" s="125"/>
     </row>
     <row r="12" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="124"/>
-      <c r="B12" s="122"/>
+      <c r="A12" s="133"/>
+      <c r="B12" s="131"/>
       <c r="C12" s="32" t="s">
         <v>57</v>
       </c>
@@ -2468,11 +2502,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B11," en el contexto de ",A5," asociado a la reserva con el identificador' ",J12,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Turno en el contexto de Agendas asociado a la reserva con el identificador' NombreTurno'.</v>
       </c>
-      <c r="S12" s="115"/>
+      <c r="S12" s="125"/>
     </row>
     <row r="13" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="125"/>
-      <c r="B13" s="122"/>
+      <c r="A13" s="134"/>
+      <c r="B13" s="131"/>
       <c r="C13" s="32" t="s">
         <v>62</v>
       </c>
@@ -2496,7 +2530,7 @@
       <c r="P13" s="32"/>
       <c r="Q13" s="32"/>
       <c r="R13" s="41"/>
-      <c r="S13" s="121"/>
+      <c r="S13" s="130"/>
     </row>
     <row r="14" spans="1:19" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -2549,75 +2583,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="99" t="str">
+      <c r="B1" s="112" t="str">
         <f>Reservas!D8</f>
         <v>Reserva-0001</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
-      <c r="R1" s="99"/>
-      <c r="S1" s="100"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
+      <c r="P1" s="112"/>
+      <c r="Q1" s="112"/>
+      <c r="R1" s="112"/>
+      <c r="S1" s="113"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="94"/>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="96"/>
+      <c r="A2" s="102"/>
+      <c r="B2" s="103"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="103"/>
+      <c r="P2" s="103"/>
+      <c r="Q2" s="103"/>
+      <c r="R2" s="103"/>
+      <c r="S2" s="104"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="114" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102" t="s">
+      <c r="B3" s="115"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="103" t="s">
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="105" t="s">
+      <c r="S3" s="118" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2673,14 +2707,14 @@
       <c r="Q4" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="R4" s="104"/>
-      <c r="S4" s="106"/>
+      <c r="R4" s="117"/>
+      <c r="S4" s="119"/>
     </row>
     <row r="5" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="131" t="s">
+      <c r="A5" s="140" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="132" t="s">
+      <c r="B5" s="141" t="s">
         <v>82</v>
       </c>
       <c r="C5" s="31" t="s">
@@ -2721,14 +2755,14 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B5,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Inmueble  en el contexto de Residentes.</v>
       </c>
-      <c r="S5" s="114" t="str">
+      <c r="S5" s="124" t="str">
         <f>B8</f>
         <v>Residente</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="131"/>
-      <c r="B6" s="133"/>
+      <c r="A6" s="140"/>
+      <c r="B6" s="142"/>
       <c r="C6" s="31" t="s">
         <v>92</v>
       </c>
@@ -2767,11 +2801,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B5," en el contexto de ",A5," asociado al residente con el identificador' ",J6,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Inmueble en el contexto de Residentes asociado al residente con el identificador' tipoInmuebleInmueble'.</v>
       </c>
-      <c r="S6" s="115"/>
+      <c r="S6" s="125"/>
     </row>
     <row r="7" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="131"/>
-      <c r="B7" s="134"/>
+      <c r="A7" s="140"/>
+      <c r="B7" s="143"/>
       <c r="C7" s="31" t="s">
         <v>93</v>
       </c>
@@ -2810,11 +2844,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B6," en el contexto de ",A6," asociado al residente con el identificador' ",J7,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' numeroViviendaInmueble'.</v>
       </c>
-      <c r="S7" s="115"/>
+      <c r="S7" s="125"/>
     </row>
     <row r="8" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="131"/>
-      <c r="B8" s="122" t="s">
+      <c r="A8" s="140"/>
+      <c r="B8" s="131" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="32" t="s">
@@ -2855,11 +2889,11 @@
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del identificador de un ",B8,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador de un Residente  en el contexto de Residentes.</v>
       </c>
-      <c r="S8" s="115"/>
+      <c r="S8" s="125"/>
     </row>
     <row r="9" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="131"/>
-      <c r="B9" s="122"/>
+      <c r="A9" s="140"/>
+      <c r="B9" s="131"/>
       <c r="C9" s="32" t="s">
         <v>57</v>
       </c>
@@ -2898,7 +2932,7 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B8," en el contexto de ",A5," asociado a la reserva con el identificador' ",J9,"'.")</f>
         <v>Atributo que contiene la información del nombre de un Residente en el contexto de Residentes asociado a la reserva con el identificador' tipoInmuebleResidente'.</v>
       </c>
-      <c r="S9" s="121"/>
+      <c r="S9" s="130"/>
     </row>
     <row r="10" spans="1:19" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
@@ -2943,29 +2977,29 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="69" t="s">
+      <c r="B1" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="70"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="78"/>
     </row>
     <row r="2" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="79" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="73"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="81"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="75"/>
-      <c r="C3" s="75"/>
-      <c r="D3" s="76"/>
+      <c r="B3" s="83"/>
+      <c r="C3" s="83"/>
+      <c r="D3" s="84"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -2982,132 +3016,132 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="79" t="s">
+      <c r="A5" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="80" t="s">
+      <c r="B5" s="88" t="s">
         <v>79</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="81" t="s">
+      <c r="D5" s="89" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="79"/>
-      <c r="B6" s="80"/>
+      <c r="A6" s="87"/>
+      <c r="B6" s="88"/>
       <c r="C6" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="81"/>
+      <c r="D6" s="89"/>
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="79"/>
-      <c r="B7" s="80"/>
+      <c r="A7" s="87"/>
+      <c r="B7" s="88"/>
       <c r="C7" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="81"/>
+      <c r="D7" s="89"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="79"/>
-      <c r="B8" s="80"/>
+      <c r="A8" s="87"/>
+      <c r="B8" s="88"/>
       <c r="C8" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="81"/>
+      <c r="D8" s="89"/>
     </row>
     <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="79"/>
-      <c r="B9" s="80"/>
+      <c r="A9" s="87"/>
+      <c r="B9" s="88"/>
       <c r="C9" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="D9" s="81"/>
+      <c r="D9" s="89"/>
     </row>
     <row r="10" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="77" t="s">
+      <c r="A10" s="85" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="78" t="s">
+      <c r="B10" s="86" t="s">
         <v>80</v>
       </c>
       <c r="C10" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="77" t="s">
+      <c r="D10" s="85" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="77"/>
-      <c r="B11" s="78"/>
+      <c r="A11" s="85"/>
+      <c r="B11" s="86"/>
       <c r="C11" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="D11" s="77"/>
+      <c r="D11" s="85"/>
     </row>
     <row r="12" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="85" t="s">
+      <c r="A12" s="93" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="82" t="s">
+      <c r="B12" s="90" t="s">
         <v>83</v>
       </c>
       <c r="C12" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="85" t="s">
+      <c r="D12" s="93" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="86"/>
-      <c r="B13" s="83"/>
+      <c r="A13" s="94"/>
+      <c r="B13" s="91"/>
       <c r="C13" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="86"/>
+      <c r="D13" s="94"/>
     </row>
     <row r="14" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="87"/>
-      <c r="B14" s="84"/>
+      <c r="A14" s="95"/>
+      <c r="B14" s="92"/>
       <c r="C14" s="27" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="87"/>
+      <c r="D14" s="95"/>
     </row>
     <row r="15" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="60" t="s">
+      <c r="A15" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="71" t="s">
         <v>63</v>
       </c>
       <c r="C15" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="66" t="s">
+      <c r="D15" s="74" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="61"/>
-      <c r="B16" s="64"/>
+      <c r="A16" s="69"/>
+      <c r="B16" s="72"/>
       <c r="C16" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="67"/>
+      <c r="D16" s="75"/>
     </row>
     <row r="17" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="62"/>
-      <c r="B17" s="65"/>
+      <c r="A17" s="70"/>
+      <c r="B17" s="73"/>
       <c r="C17" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="68"/>
+      <c r="D17" s="76"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -3179,50 +3213,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="88" t="str">
+      <c r="B1" s="96" t="str">
         <f>Contextos!B5</f>
         <v xml:space="preserve"> Conjuntos residenciales</v>
       </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="89"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="97"/>
     </row>
     <row r="2" spans="1:6" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="90" t="str">
+      <c r="B2" s="98" t="str">
         <f>Contextos!D5</f>
         <v>Contexto cuya motivación es Gestionar la estructura física y los recursos disponibles en cada conjunto residencial. Aquí se manejan los datos sobre qué conjuntos existen, dónde están ubicados, qué recursos ofrecen según una Agenda con respectivos turnos para cada zona.</v>
       </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="91"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="99"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="92" t="str">
+      <c r="B3" s="100" t="str">
         <f>Contextos!A5</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="93"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="101"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="94" t="s">
+      <c r="A4" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="95"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="96"/>
+      <c r="B4" s="103"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="104"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -3231,14 +3265,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="97" t="s">
+      <c r="C5" s="105" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="97" t="s">
+      <c r="D5" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="97"/>
-      <c r="F5" s="98" t="s">
+      <c r="E5" s="105"/>
+      <c r="F5" s="106" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3249,10 +3283,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="97"/>
-      <c r="E6" s="97"/>
-      <c r="F6" s="98"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="106"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -3261,14 +3295,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="97"/>
+      <c r="C7" s="105"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="98"/>
+      <c r="F7" s="106"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
@@ -3402,50 +3436,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="88" t="str">
+      <c r="B1" s="96" t="str">
         <f>Contextos!B10</f>
         <v>Residentes</v>
       </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="89"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="97"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="90" t="str">
+      <c r="B2" s="98" t="str">
         <f>Contextos!D10</f>
         <v>Contexto cuya motivación es encargarce de manejar la información de los residentes, incluidas sus identificaciones, contacto, y la relación entre el residente y su residencia dentro del conjunto.</v>
       </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="91"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="99"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="92" t="str">
+      <c r="B3" s="100" t="str">
         <f>Contextos!A10</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="93"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="101"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="94" t="s">
+      <c r="A4" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="95"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="96"/>
+      <c r="B4" s="103"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="104"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -3454,14 +3488,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="97" t="s">
+      <c r="C5" s="105" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="97" t="s">
+      <c r="D5" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="97"/>
-      <c r="F5" s="98" t="s">
+      <c r="E5" s="105"/>
+      <c r="F5" s="106" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3472,10 +3506,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="97"/>
-      <c r="E6" s="97"/>
-      <c r="F6" s="98"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="106"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -3484,14 +3518,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="97"/>
+      <c r="C7" s="105"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="98"/>
+      <c r="F7" s="106"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
@@ -3546,7 +3580,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59635CF3-0DE6-45E6-A198-1E7042F5E8F9}">
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" style="13" bestFit="1" customWidth="1"/>
@@ -3575,75 +3609,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="99" t="str">
+      <c r="B1" s="112" t="str">
         <f>Residentes!D8</f>
         <v>Residente Inmueble-0001</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
-      <c r="R1" s="99"/>
-      <c r="S1" s="100"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
+      <c r="P1" s="112"/>
+      <c r="Q1" s="112"/>
+      <c r="R1" s="112"/>
+      <c r="S1" s="113"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="94"/>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="96"/>
+      <c r="A2" s="102"/>
+      <c r="B2" s="103"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="103"/>
+      <c r="P2" s="103"/>
+      <c r="Q2" s="103"/>
+      <c r="R2" s="103"/>
+      <c r="S2" s="104"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="114" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102" t="s">
+      <c r="B3" s="115"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="103" t="s">
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="105" t="s">
+      <c r="S3" s="118" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3699,17 +3733,17 @@
       <c r="Q4" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="R4" s="104"/>
-      <c r="S4" s="106"/>
+      <c r="R4" s="117"/>
+      <c r="S4" s="119"/>
     </row>
     <row r="5" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="108" t="s">
+      <c r="A5" s="107" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="140" t="s">
+      <c r="B5" s="145" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="139" t="s">
+      <c r="C5" s="61" t="s">
         <v>93</v>
       </c>
       <c r="D5" s="51" t="s">
@@ -3743,287 +3777,435 @@
       <c r="O5" s="51"/>
       <c r="P5" s="51"/>
       <c r="Q5" s="52"/>
-      <c r="R5" s="143" t="str">
+      <c r="R5" s="62" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C5," del objeto dominio ",B5,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del numeroVivienda del objeto dominio Inmueble  en el contexto de Conjuntos Residenciales.</v>
       </c>
-      <c r="S5" s="141" t="s">
+      <c r="S5" s="109" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="108"/>
-      <c r="B6" s="110" t="s">
+    <row r="6" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="107"/>
+      <c r="B6" s="146"/>
+      <c r="C6" s="144" t="s">
         <v>100</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="51"/>
+      <c r="K6" s="51"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="51"/>
+      <c r="N6" s="51"/>
+      <c r="O6" s="51"/>
+      <c r="P6" s="51"/>
+      <c r="Q6" s="52"/>
+      <c r="R6" s="62"/>
+      <c r="S6" s="109"/>
+    </row>
+    <row r="7" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="107"/>
+      <c r="B7" s="147" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="50" t="s">
         <v>55</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D7" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="E6" s="31">
+      <c r="E7" s="31">
         <v>32</v>
       </c>
-      <c r="F6" s="31">
+      <c r="F7" s="31">
         <v>32</v>
-      </c>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31" t="str">
-        <f>_xlfn.CONCAT(C6,$B$6)</f>
-        <v>identificadorTipoInmueble</v>
-      </c>
-      <c r="K6" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="L6" s="31" t="s">
-        <v>56</v>
-      </c>
-      <c r="M6" s="31">
-        <v>32</v>
-      </c>
-      <c r="N6" s="31">
-        <v>32</v>
-      </c>
-      <c r="O6" s="31"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="53"/>
-      <c r="R6" s="144" t="str">
-        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C6," del objeto dominio ",B6,"  en el contexto de ",A5,".")</f>
-        <v>Atributo que contiene la informacion del identificador del objeto dominio TipoInmueble  en el contexto de Conjuntos Residenciales.</v>
-      </c>
-      <c r="S6" s="141"/>
-    </row>
-    <row r="7" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="108"/>
-      <c r="B7" s="110"/>
-      <c r="C7" s="50" t="s">
-        <v>57</v>
-      </c>
-      <c r="D7" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" s="31">
-        <v>1</v>
-      </c>
-      <c r="F7" s="31">
-        <v>50</v>
       </c>
       <c r="G7" s="31"/>
       <c r="H7" s="31"/>
       <c r="I7" s="31"/>
       <c r="J7" s="31" t="str">
-        <f>_xlfn.CONCAT(C7,$B$6)</f>
-        <v>nombreTipoInmueble</v>
-      </c>
-      <c r="K7" s="31"/>
+        <f>_xlfn.CONCAT(C7,$B$7)</f>
+        <v>identificadorTipoInmueble</v>
+      </c>
+      <c r="K7" s="31" t="s">
+        <v>59</v>
+      </c>
       <c r="L7" s="31" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="M7" s="31">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="N7" s="31">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="O7" s="31"/>
       <c r="P7" s="31"/>
       <c r="Q7" s="53"/>
-      <c r="R7" s="144" t="str">
+      <c r="R7" s="63" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C7," del objeto dominio ",B7,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del identificador del objeto dominio TipoInmueble  en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S7" s="109"/>
+    </row>
+    <row r="8" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="107"/>
+      <c r="B8" s="148"/>
+      <c r="C8" s="50" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="31">
+        <v>1</v>
+      </c>
+      <c r="F8" s="31">
+        <v>50</v>
+      </c>
+      <c r="G8" s="31"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="31" t="str">
+        <f>_xlfn.CONCAT(C8,$B$7)</f>
+        <v>nombreTipoInmueble</v>
+      </c>
+      <c r="K8" s="31"/>
+      <c r="L8" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="M8" s="31">
+        <v>1</v>
+      </c>
+      <c r="N8" s="31">
+        <v>50</v>
+      </c>
+      <c r="O8" s="31"/>
+      <c r="P8" s="31"/>
+      <c r="Q8" s="53"/>
+      <c r="R8" s="63" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C8," del objeto dominio ",B8,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del nombre del objeto dominio   en el contexto de Conjuntos Residenciales.</v>
       </c>
-      <c r="S7" s="141"/>
-    </row>
-    <row r="8" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="108"/>
-      <c r="B8" s="135" t="s">
+      <c r="S8" s="109"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="107"/>
+      <c r="B9" s="149"/>
+      <c r="C9" s="50" t="s">
         <v>81</v>
       </c>
-      <c r="C8" s="136" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="31"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="53"/>
+      <c r="R9" s="63"/>
+      <c r="S9" s="109"/>
+    </row>
+    <row r="10" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="107"/>
+      <c r="B10" s="150" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="137" t="s">
+      <c r="D10" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="137">
+      <c r="E10" s="59">
         <v>32</v>
       </c>
-      <c r="F8" s="137">
+      <c r="F10" s="59">
         <v>32</v>
       </c>
-      <c r="G8" s="137"/>
-      <c r="H8" s="137"/>
-      <c r="I8" s="137"/>
-      <c r="J8" s="137" t="str">
-        <f>_xlfn.CONCAT(C8,$B$6)</f>
+      <c r="G10" s="59"/>
+      <c r="H10" s="59"/>
+      <c r="I10" s="59"/>
+      <c r="J10" s="59" t="str">
+        <f>_xlfn.CONCAT(C10,$B$7)</f>
         <v>identificadorTipoInmueble</v>
       </c>
-      <c r="K8" s="137" t="s">
+      <c r="K10" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="L8" s="137" t="s">
+      <c r="L10" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="M8" s="137">
+      <c r="M10" s="59">
         <v>32</v>
       </c>
-      <c r="N8" s="137">
+      <c r="N10" s="59">
         <v>32</v>
       </c>
-      <c r="O8" s="137"/>
-      <c r="P8" s="137"/>
-      <c r="Q8" s="138"/>
-      <c r="R8" s="145" t="str">
-        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C8," del objeto dominio ",B8,"  en el contexto de ",A5,".")</f>
-        <v>Atributo que contiene la informacion del identificador del objeto dominio ZonaInmueble  en el contexto de Conjuntos Residenciales.</v>
-      </c>
-      <c r="S8" s="141"/>
-    </row>
-    <row r="9" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="108"/>
-      <c r="B9" s="135"/>
-      <c r="C9" s="136" t="s">
+      <c r="O10" s="59"/>
+      <c r="P10" s="59"/>
+      <c r="Q10" s="60"/>
+      <c r="R10" s="64" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C10," del objeto dominio ",B10,"  en el contexto de ",A3,".")</f>
+        <v>Atributo que contiene la informacion del identificador del objeto dominio ZonaInmueble  en el contexto de Caracterización Origen.</v>
+      </c>
+      <c r="S10" s="109"/>
+    </row>
+    <row r="11" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="107"/>
+      <c r="B11" s="152"/>
+      <c r="C11" s="58" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" s="59"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="59"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="59"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="59" t="str">
+        <f>_xlfn.CONCAT(C11,$B$7)</f>
+        <v>TipoZonaInmuebleTipoInmueble</v>
+      </c>
+      <c r="K11" s="59"/>
+      <c r="L11" s="59"/>
+      <c r="M11" s="59"/>
+      <c r="N11" s="59"/>
+      <c r="O11" s="59"/>
+      <c r="P11" s="59"/>
+      <c r="Q11" s="60"/>
+      <c r="R11" s="64" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C11," del objeto dominio ",B11,"  en el contexto de ",A3,".")</f>
+        <v>Atributo que contiene la informacion del TipoZonaInmueble del objeto dominio   en el contexto de Caracterización Origen.</v>
+      </c>
+      <c r="S11" s="109"/>
+    </row>
+    <row r="12" spans="1:19" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="107"/>
+      <c r="B12" s="151"/>
+      <c r="C12" s="58" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="59"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59" t="str">
+        <f>_xlfn.CONCAT(C12,$B$7)</f>
+        <v>ConjuntoResidencialTipoInmueble</v>
+      </c>
+      <c r="K12" s="59"/>
+      <c r="L12" s="59"/>
+      <c r="M12" s="59"/>
+      <c r="N12" s="59"/>
+      <c r="O12" s="59"/>
+      <c r="P12" s="59"/>
+      <c r="Q12" s="60"/>
+      <c r="R12" s="64"/>
+      <c r="S12" s="109"/>
+    </row>
+    <row r="13" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="107"/>
+      <c r="B13" s="150" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="59" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="59">
+        <v>32</v>
+      </c>
+      <c r="F13" s="59">
+        <v>32</v>
+      </c>
+      <c r="G13" s="59"/>
+      <c r="H13" s="59"/>
+      <c r="I13" s="59"/>
+      <c r="J13" s="59" t="str">
+        <f>_xlfn.CONCAT(C13,$B$7)</f>
+        <v>identificadorTipoInmueble</v>
+      </c>
+      <c r="K13" s="59" t="s">
+        <v>59</v>
+      </c>
+      <c r="L13" s="59" t="s">
+        <v>56</v>
+      </c>
+      <c r="M13" s="59">
+        <v>32</v>
+      </c>
+      <c r="N13" s="59">
+        <v>32</v>
+      </c>
+      <c r="O13" s="59"/>
+      <c r="P13" s="59"/>
+      <c r="Q13" s="60"/>
+      <c r="R13" s="64" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C13," del objeto dominio ",B13,"  en el contexto de ",A5,".")</f>
+        <v>Atributo que contiene la informacion del identificador del objeto dominio TipoZonaInmueble  en el contexto de Conjuntos Residenciales.</v>
+      </c>
+      <c r="S13" s="109"/>
+    </row>
+    <row r="14" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="107"/>
+      <c r="B14" s="152"/>
+      <c r="C14" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="137" t="s">
+      <c r="D14" s="59" t="s">
         <v>58</v>
       </c>
-      <c r="E9" s="137">
+      <c r="E14" s="59">
         <v>1</v>
       </c>
-      <c r="F9" s="137">
+      <c r="F14" s="59">
         <v>50</v>
       </c>
-      <c r="G9" s="137"/>
-      <c r="H9" s="137"/>
-      <c r="I9" s="137"/>
-      <c r="J9" s="137" t="str">
-        <f>_xlfn.CONCAT(C9,$B$6)</f>
+      <c r="G14" s="59"/>
+      <c r="H14" s="59"/>
+      <c r="I14" s="59"/>
+      <c r="J14" s="59" t="str">
+        <f>_xlfn.CONCAT(C14,$B$7)</f>
         <v>nombreTipoInmueble</v>
       </c>
-      <c r="K9" s="137"/>
-      <c r="L9" s="137" t="s">
+      <c r="K14" s="59"/>
+      <c r="L14" s="59" t="s">
         <v>58</v>
       </c>
-      <c r="M9" s="137">
+      <c r="M14" s="59">
         <v>1</v>
       </c>
-      <c r="N9" s="137">
+      <c r="N14" s="59">
         <v>50</v>
       </c>
-      <c r="O9" s="137"/>
-      <c r="P9" s="137"/>
-      <c r="Q9" s="138"/>
-      <c r="R9" s="145" t="str">
-        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C9," del objeto dominio ",B9,"  en el contexto de ",A5,".")</f>
+      <c r="O14" s="59"/>
+      <c r="P14" s="59"/>
+      <c r="Q14" s="60"/>
+      <c r="R14" s="64" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C14," del objeto dominio ",B14,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del nombre del objeto dominio   en el contexto de Conjuntos Residenciales.</v>
       </c>
-      <c r="S9" s="141"/>
-    </row>
-    <row r="10" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="108"/>
-      <c r="B10" s="111" t="s">
+      <c r="S14" s="109"/>
+    </row>
+    <row r="15" spans="1:19" ht="44.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="107"/>
+      <c r="B15" s="111" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C15" s="32" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D15" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="32">
+      <c r="E15" s="32">
         <v>32</v>
       </c>
-      <c r="F10" s="32">
+      <c r="F15" s="32">
         <v>32</v>
       </c>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="32" t="str">
-        <f>_xlfn.CONCAT(C6,$B$10)</f>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32" t="str">
+        <f>_xlfn.CONCAT(C7,$B$15)</f>
         <v>identificadorConjuntoResidencial</v>
       </c>
-      <c r="K10" s="32" t="s">
+      <c r="K15" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="L10" s="32" t="s">
+      <c r="L15" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="M10" s="32">
+      <c r="M15" s="32">
         <v>32</v>
       </c>
-      <c r="N10" s="32">
+      <c r="N15" s="32">
         <v>32</v>
       </c>
-      <c r="O10" s="32"/>
-      <c r="P10" s="32"/>
-      <c r="Q10" s="54"/>
-      <c r="R10" s="146" t="str">
-        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C10," del objeto dominio ",B10,"  en el contexto de ",A5,".")</f>
+      <c r="O15" s="32"/>
+      <c r="P15" s="32"/>
+      <c r="Q15" s="54"/>
+      <c r="R15" s="65" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C15," del objeto dominio ",B15,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del identificador del objeto dominio ConjuntoResidencial  en el contexto de Conjuntos Residenciales.</v>
       </c>
-      <c r="S10" s="141"/>
-    </row>
-    <row r="11" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="109"/>
-      <c r="B11" s="111"/>
-      <c r="C11" s="32" t="s">
+      <c r="S15" s="109"/>
+    </row>
+    <row r="16" spans="1:19" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="108"/>
+      <c r="B16" s="111"/>
+      <c r="C16" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="32" t="s">
+      <c r="D16" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="32">
+      <c r="E16" s="32">
         <v>1</v>
       </c>
-      <c r="F11" s="32">
+      <c r="F16" s="32">
         <v>50</v>
       </c>
-      <c r="G11" s="32"/>
-      <c r="H11" s="32"/>
-      <c r="I11" s="32"/>
-      <c r="J11" s="32" t="str">
-        <f>_xlfn.CONCAT(C7,$B$10)</f>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32" t="str">
+        <f>_xlfn.CONCAT(C8,$B$15)</f>
         <v>nombreConjuntoResidencial</v>
       </c>
-      <c r="K11" s="32" t="s">
+      <c r="K16" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="L11" s="32" t="s">
+      <c r="L16" s="32" t="s">
         <v>58</v>
       </c>
-      <c r="M11" s="32">
+      <c r="M16" s="32">
         <v>1</v>
       </c>
-      <c r="N11" s="32">
+      <c r="N16" s="32">
         <v>50</v>
       </c>
-      <c r="O11" s="32"/>
-      <c r="P11" s="32"/>
-      <c r="Q11" s="54"/>
-      <c r="R11" s="146" t="str">
-        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C11," del objeto dominio ",B11,"  en el contexto de ",A5,".")</f>
+      <c r="O16" s="32"/>
+      <c r="P16" s="32"/>
+      <c r="Q16" s="54"/>
+      <c r="R16" s="65" t="str">
+        <f>_xlfn.CONCAT("Atributo que contiene la informacion del ",C16," del objeto dominio ",B16,"  en el contexto de ",A5,".")</f>
         <v>Atributo que contiene la informacion del nombre del objeto dominio   en el contexto de Conjuntos Residenciales.</v>
       </c>
-      <c r="S11" s="142"/>
+      <c r="S16" s="110"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A5:A11"/>
-    <mergeCell ref="S5:S11"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B8:B9"/>
+  <mergeCells count="13">
     <mergeCell ref="B1:S1"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="J3:Q3"/>
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
+    <mergeCell ref="A5:A16"/>
+    <mergeCell ref="S5:S16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B10:B12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4046,50 +4228,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="88" t="str">
+      <c r="B1" s="96" t="str">
         <f>Contextos!B12</f>
         <v>Agendas</v>
       </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="89"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="97"/>
     </row>
     <row r="2" spans="1:6" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="90" t="str">
+      <c r="B2" s="98" t="str">
         <f>Contextos!D12</f>
         <v>Contexto cuya motivación es la de gestionar la estructura de la agenda que va a tener una zona común durante un un tiempo estimado y sus diferentes turnos.</v>
       </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="91"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="99"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="92" t="str">
+      <c r="B3" s="100" t="str">
         <f>Contextos!A12</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="93"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="101"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="94" t="s">
+      <c r="A4" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="95"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="96"/>
+      <c r="B4" s="103"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="104"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -4098,14 +4280,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="97" t="s">
+      <c r="C5" s="105" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="97" t="s">
+      <c r="D5" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="97"/>
-      <c r="F5" s="98" t="s">
+      <c r="E5" s="105"/>
+      <c r="F5" s="106" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4116,10 +4298,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="97"/>
-      <c r="E6" s="97"/>
-      <c r="F6" s="98"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="106"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -4128,14 +4310,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="97"/>
+      <c r="C7" s="105"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="98"/>
+      <c r="F7" s="106"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
@@ -4241,75 +4423,75 @@
       <c r="A1" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="99" t="str">
+      <c r="B1" s="112" t="str">
         <f>Agendas!D8</f>
         <v>Agenda ZonaComun-0001</v>
       </c>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
-      <c r="J1" s="99"/>
-      <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99"/>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="99"/>
-      <c r="R1" s="99"/>
-      <c r="S1" s="100"/>
+      <c r="C1" s="112"/>
+      <c r="D1" s="112"/>
+      <c r="E1" s="112"/>
+      <c r="F1" s="112"/>
+      <c r="G1" s="112"/>
+      <c r="H1" s="112"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="112"/>
+      <c r="L1" s="112"/>
+      <c r="M1" s="112"/>
+      <c r="N1" s="112"/>
+      <c r="O1" s="112"/>
+      <c r="P1" s="112"/>
+      <c r="Q1" s="112"/>
+      <c r="R1" s="112"/>
+      <c r="S1" s="113"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="94"/>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
-      <c r="P2" s="95"/>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="95"/>
-      <c r="S2" s="96"/>
+      <c r="A2" s="102"/>
+      <c r="B2" s="103"/>
+      <c r="C2" s="103"/>
+      <c r="D2" s="103"/>
+      <c r="E2" s="103"/>
+      <c r="F2" s="103"/>
+      <c r="G2" s="103"/>
+      <c r="H2" s="103"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="103"/>
+      <c r="L2" s="103"/>
+      <c r="M2" s="103"/>
+      <c r="N2" s="103"/>
+      <c r="O2" s="103"/>
+      <c r="P2" s="103"/>
+      <c r="Q2" s="103"/>
+      <c r="R2" s="103"/>
+      <c r="S2" s="104"/>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="114" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="102"/>
-      <c r="C3" s="102"/>
-      <c r="D3" s="102"/>
-      <c r="E3" s="102"/>
-      <c r="F3" s="102"/>
-      <c r="G3" s="102"/>
-      <c r="H3" s="102"/>
-      <c r="I3" s="102"/>
-      <c r="J3" s="102" t="s">
+      <c r="B3" s="115"/>
+      <c r="C3" s="115"/>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="115"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
+      <c r="J3" s="115" t="s">
         <v>43</v>
       </c>
-      <c r="K3" s="102"/>
-      <c r="L3" s="102"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="102"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="102"/>
-      <c r="Q3" s="102"/>
-      <c r="R3" s="103" t="s">
+      <c r="K3" s="115"/>
+      <c r="L3" s="115"/>
+      <c r="M3" s="115"/>
+      <c r="N3" s="115"/>
+      <c r="O3" s="115"/>
+      <c r="P3" s="115"/>
+      <c r="Q3" s="115"/>
+      <c r="R3" s="116" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="105" t="s">
+      <c r="S3" s="118" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4366,13 +4548,13 @@
         <v>52</v>
       </c>
       <c r="R4" s="120"/>
-      <c r="S4" s="106"/>
+      <c r="S4" s="119"/>
     </row>
     <row r="5" spans="1:19" ht="28.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="107" t="s">
+      <c r="A5" s="121" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="116" t="s">
+      <c r="B5" s="126" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="51" t="s">
@@ -4409,17 +4591,17 @@
       <c r="O5" s="51"/>
       <c r="P5" s="51"/>
       <c r="Q5" s="51"/>
-      <c r="R5" s="112" t="str">
+      <c r="R5" s="122" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B7," en el contexto de ",A5," asociado al residente con el identificador' ",J9,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de Conjuntos Residenciales asociado al residente con el identificador' unidadTiempoUsoZonaComun'.</v>
       </c>
-      <c r="S5" s="114" t="s">
+      <c r="S5" s="124" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="108"/>
-      <c r="B6" s="117"/>
+      <c r="A6" s="107"/>
+      <c r="B6" s="127"/>
       <c r="C6" s="51" t="s">
         <v>4</v>
       </c>
@@ -4454,12 +4636,12 @@
       <c r="O6" s="51"/>
       <c r="P6" s="51"/>
       <c r="Q6" s="51"/>
-      <c r="R6" s="113"/>
-      <c r="S6" s="115"/>
+      <c r="R6" s="123"/>
+      <c r="S6" s="125"/>
     </row>
     <row r="7" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="108"/>
-      <c r="B7" s="117"/>
+      <c r="A7" s="107"/>
+      <c r="B7" s="127"/>
       <c r="C7" s="51" t="s">
         <v>97</v>
       </c>
@@ -4482,15 +4664,15 @@
       <c r="O7" s="51"/>
       <c r="P7" s="51"/>
       <c r="Q7" s="51"/>
-      <c r="R7" s="112" t="str">
+      <c r="R7" s="122" t="str">
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B9," en el contexto de ",A7," asociado al residente con el identificador' ",J11,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' nombreConjuntoResidencial'.</v>
       </c>
-      <c r="S7" s="115"/>
+      <c r="S7" s="125"/>
     </row>
     <row r="8" spans="1:19" ht="30.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="108"/>
-      <c r="B8" s="117"/>
+      <c r="A8" s="107"/>
+      <c r="B8" s="127"/>
       <c r="C8" s="51" t="s">
         <v>98</v>
       </c>
@@ -4513,12 +4695,12 @@
       <c r="O8" s="51"/>
       <c r="P8" s="51"/>
       <c r="Q8" s="51"/>
-      <c r="R8" s="119"/>
-      <c r="S8" s="115"/>
+      <c r="R8" s="129"/>
+      <c r="S8" s="125"/>
     </row>
     <row r="9" spans="1:19" ht="61.8" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="108"/>
-      <c r="B9" s="118"/>
+      <c r="A9" s="107"/>
+      <c r="B9" s="128"/>
       <c r="C9" s="51" t="s">
         <v>99</v>
       </c>
@@ -4545,10 +4727,10 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B11," en el contexto de ",A9," asociado al residente con el identificador' ",J13,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado al residente con el identificador' '.</v>
       </c>
-      <c r="S9" s="115"/>
+      <c r="S9" s="125"/>
     </row>
     <row r="10" spans="1:19" ht="60.6" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="108"/>
+      <c r="A10" s="107"/>
       <c r="B10" s="111" t="s">
         <v>61</v>
       </c>
@@ -4590,10 +4772,10 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B10," en el contexto de ",A10," asociado a la reserva con el identificador' ",J10,"'.")</f>
         <v>Atributo que contiene la información del nombre de un ConjuntoResidencial en el contexto de  asociado a la reserva con el identificador' identificadorConjuntoResidencial'.</v>
       </c>
-      <c r="S10" s="115"/>
+      <c r="S10" s="125"/>
     </row>
     <row r="11" spans="1:19" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="109"/>
+      <c r="A11" s="108"/>
       <c r="B11" s="111"/>
       <c r="C11" s="32" t="s">
         <v>57</v>
@@ -4633,22 +4815,22 @@
         <f>_xlfn.CONCAT("Atributo que contiene la información del nombre de un ",B11," en el contexto de ",A11," asociado a la reserva con el identificador' ",J11,"'.")</f>
         <v>Atributo que contiene la información del nombre de un  en el contexto de  asociado a la reserva con el identificador' nombreConjuntoResidencial'.</v>
       </c>
-      <c r="S11" s="115"/>
+      <c r="S11" s="125"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A5:A11"/>
+    <mergeCell ref="R5:R6"/>
+    <mergeCell ref="S5:S11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B5:B9"/>
+    <mergeCell ref="R7:R8"/>
     <mergeCell ref="B1:S1"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="J3:Q3"/>
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:S4"/>
-    <mergeCell ref="A5:A11"/>
-    <mergeCell ref="R5:R6"/>
-    <mergeCell ref="S5:S11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="B5:B9"/>
-    <mergeCell ref="R7:R8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4672,50 +4854,50 @@
       <c r="A1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="88" t="str">
+      <c r="B1" s="96" t="str">
         <f>Contextos!B15</f>
         <v>Reservas</v>
       </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="89"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="97"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="90" t="str">
+      <c r="B2" s="98" t="str">
         <f>Contextos!D15</f>
         <v>Contexto cuya intención enfocarse en la gestión del proceso de reservas de los recursos, incluyendo la disponibilidad de los recursos y las reservas que los residentes realizan.</v>
       </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="91"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="99"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="92" t="str">
+      <c r="B3" s="100" t="str">
         <f>Contextos!A15</f>
         <v>Core/Básico</v>
       </c>
-      <c r="C3" s="92"/>
-      <c r="D3" s="92"/>
-      <c r="E3" s="92"/>
-      <c r="F3" s="93"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="101"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="94" t="s">
+      <c r="A4" s="102" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="95"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="96"/>
+      <c r="B4" s="103"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="104"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
@@ -4724,14 +4906,14 @@
       <c r="B5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="97" t="s">
+      <c r="C5" s="105" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="97" t="s">
+      <c r="D5" s="105" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="97"/>
-      <c r="F5" s="98" t="s">
+      <c r="E5" s="105"/>
+      <c r="F5" s="106" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4742,10 +4924,10 @@
       <c r="B6" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="97"/>
-      <c r="E6" s="97"/>
-      <c r="F6" s="98"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="106"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
@@ -4754,14 +4936,14 @@
       <c r="B7" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="97"/>
+      <c r="C7" s="105"/>
       <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
       <c r="E7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="F7" s="98"/>
+      <c r="F7" s="106"/>
     </row>
     <row r="8" spans="1:6" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">

</xml_diff>